<commit_message>
Fase 163 (3): Llamadas Unicas: el asesor no es obligatorio; sin asesor = abandonada; una sola barra si no hay abandonadas (v1.62.0)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_LLAMADAS_UNICAS.xlsx
+++ b/server/plantillas/PLANTILLA_LLAMADAS_UNICAS.xlsx
@@ -448,7 +448,7 @@
         <v>De dónde sale</v>
       </c>
       <c r="B2" t="str">
-        <v>Wolkvox: Reportes → CDR → "1. Detalle de las llamadas", solo las de ingreso (sin las de salida).</v>
+        <v>Wolkvox, dos reportes en una sola hoja: las CONTESTADAS del CDR → "1. Detalle de las llamadas" (solo las de ingreso, con asesor) y las ABANDONADAS de "Skill y servicios → 2. Detalle llamadas abandonadas" (skill, teléfono y día, con AGENT_NAME vacío).</v>
       </c>
     </row>
     <row r="3">
@@ -508,7 +508,7 @@
         <v>Sí</v>
       </c>
       <c r="C9" t="str">
-        <v>Asesor que atendió.</v>
+        <v>Asesor que atendió. Vacío en las abandonadas (el reporte de abandonadas no trae asesor): una fila sin asesor cuenta como abandonada.</v>
       </c>
       <c r="D9" t="str">
         <v>Asesor Ejemplo Uno</v>

</xml_diff>